<commit_message>
Update Polymarket 30-day dashboard data
</commit_message>
<xml_diff>
--- a/docs/data/kalshi_cumulative_topic_share.xlsx
+++ b/docs/data/kalshi_cumulative_topic_share.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="current" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="history" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="current" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="history" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -488,13 +488,13 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>412447.74</v>
+        <v>267605.81</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>93.02271253000001</v>
+        <v>86.81310058</v>
       </c>
       <c r="E2" t="n">
-        <v>383</v>
+        <v>340</v>
       </c>
     </row>
     <row r="3">
@@ -509,13 +509,13 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>28521.45</v>
+        <v>39275.92</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>6.43267592</v>
+        <v>12.74136908</v>
       </c>
       <c r="E3" t="n">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="4">
@@ -526,17 +526,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Business/Economy</t>
+          <t>Geopolitics</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>2272.72</v>
+        <v>894.3099999999999</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>0.5125851300000001</v>
+        <v>0.2901201</v>
       </c>
       <c r="E4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5">
@@ -551,13 +551,13 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>142</v>
+        <v>479.06</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>0.03202642</v>
+        <v>0.15541024</v>
       </c>
       <c r="E5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6">
@@ -572,13 +572,13 @@
         </is>
       </c>
       <c r="C6" s="5" t="n">
-        <v>443383.91</v>
+        <v>308255.1</v>
       </c>
       <c r="D6" s="6" t="n">
         <v>100</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>457</v>
+        <v>416</v>
       </c>
     </row>
   </sheetData>
@@ -637,17 +637,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Business/Economy</t>
+          <t>Geopolitics</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>2272.72</v>
+        <v>894.3099999999999</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0.5125851300000001</v>
+        <v>0.2901201</v>
       </c>
       <c r="E2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3">
@@ -662,13 +662,13 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>412447.74</v>
+        <v>267605.81</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>93.02271253000001</v>
+        <v>86.81310058</v>
       </c>
       <c r="E3" t="n">
-        <v>383</v>
+        <v>340</v>
       </c>
     </row>
     <row r="4">
@@ -683,13 +683,13 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>142</v>
+        <v>479.06</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>0.03202642</v>
+        <v>0.15541024</v>
       </c>
       <c r="E4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5">
@@ -704,13 +704,13 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>28521.45</v>
+        <v>39275.92</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>6.43267592</v>
+        <v>12.74136908</v>
       </c>
       <c r="E5" t="n">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
   </sheetData>

</xml_diff>